<commit_message>
configure parameterized browers and env
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Selenium\seleniumtests\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FBA9CFB-7CFE-47DE-A0CD-69160E6BB23F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29649315-1120-400A-88ED-F191603514E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2280" yWindow="2280" windowWidth="14400" windowHeight="7270" xr2:uid="{8A7B9094-5F1A-4583-BBB8-AA626BD128D4}"/>
   </bookViews>
@@ -428,19 +428,19 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
+      <c r="B2">
+        <v>111</v>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3">
-        <v>111</v>
+        <v>111111</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>
@@ -450,8 +450,8 @@
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
-        <v>111111</v>
+      <c r="B4" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C4" t="b">
         <v>0</v>
@@ -459,10 +459,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{16AB517E-34F2-424C-AFAC-C129FF331394}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{B8E1E6B5-EBD7-400C-BEB0-3965EB459AE5}"/>
-    <hyperlink ref="A3" r:id="rId3" xr:uid="{628FA617-5A4E-43D1-A02B-C2EE7AC97F45}"/>
-    <hyperlink ref="A4" r:id="rId4" xr:uid="{D583CBC0-FF9C-4BD8-A24C-8894CC58B63E}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{628FA617-5A4E-43D1-A02B-C2EE7AC97F45}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{D583CBC0-FF9C-4BD8-A24C-8894CC58B63E}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{DDFA63D9-1EDB-4EBB-A98A-A549244B0AF8}"/>
+    <hyperlink ref="B4" r:id="rId4" xr:uid="{5CF12BA3-5F39-43E6-9A1D-6B23627379A8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId5"/>

</xml_diff>